<commit_message>
Cleared blank spreadsheets for week 2 examples
</commit_message>
<xml_diff>
--- a/Module 1/Week 2 - Investment returns, portfolios, and indexes/Example from textbook p48.xlsx
+++ b/Module 1/Week 2 - Investment returns, portfolios, and indexes/Example from textbook p48.xlsx
@@ -5,14 +5,14 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="4"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Table 2_2" sheetId="1" state="visible" r:id="rId2"/>
-    <sheet name="Example 1 - Price weighting" sheetId="2" state="visible" r:id="rId3"/>
-    <sheet name="Example 2 - Equal weighting" sheetId="3" state="visible" r:id="rId4"/>
-    <sheet name="Example 3 - Value weighting" sheetId="4" state="visible" r:id="rId5"/>
-    <sheet name="Example 4 - Change in a value-w" sheetId="5" state="visible" r:id="rId6"/>
+    <sheet name="Table 2_2" sheetId="1" state="visible" r:id="rId3"/>
+    <sheet name="Example 1 - Price weighting" sheetId="2" state="visible" r:id="rId4"/>
+    <sheet name="Example 2 - Equal weighting" sheetId="3" state="visible" r:id="rId5"/>
+    <sheet name="Example 3 - Value weighting" sheetId="4" state="visible" r:id="rId6"/>
+    <sheet name="Example 4 - Change in a value-w" sheetId="5" state="visible" r:id="rId7"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
   <extLst>
@@ -168,12 +168,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="5">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="[$$-409]#,##0.00;[RED]\-[$$-409]#,##0.00"/>
-    <numFmt numFmtId="166" formatCode="General"/>
-    <numFmt numFmtId="167" formatCode="0.00%"/>
-    <numFmt numFmtId="168" formatCode="0.000"/>
+    <numFmt numFmtId="166" formatCode="0.00%"/>
+    <numFmt numFmtId="167" formatCode="0.000"/>
   </numFmts>
   <fonts count="7">
     <font>
@@ -261,52 +260,56 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="166" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -322,85 +325,191 @@
 </styleSheet>
 </file>
 
+<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office">
+  <a:themeElements>
+    <a:clrScheme name="LibreOffice">
+      <a:dk1>
+        <a:srgbClr val="000000"/>
+      </a:dk1>
+      <a:lt1>
+        <a:srgbClr val="ffffff"/>
+      </a:lt1>
+      <a:dk2>
+        <a:srgbClr val="000000"/>
+      </a:dk2>
+      <a:lt2>
+        <a:srgbClr val="ffffff"/>
+      </a:lt2>
+      <a:accent1>
+        <a:srgbClr val="18a303"/>
+      </a:accent1>
+      <a:accent2>
+        <a:srgbClr val="0369a3"/>
+      </a:accent2>
+      <a:accent3>
+        <a:srgbClr val="a33e03"/>
+      </a:accent3>
+      <a:accent4>
+        <a:srgbClr val="8e03a3"/>
+      </a:accent4>
+      <a:accent5>
+        <a:srgbClr val="c99c00"/>
+      </a:accent5>
+      <a:accent6>
+        <a:srgbClr val="c9211e"/>
+      </a:accent6>
+      <a:hlink>
+        <a:srgbClr val="0000ee"/>
+      </a:hlink>
+      <a:folHlink>
+        <a:srgbClr val="551a8b"/>
+      </a:folHlink>
+    </a:clrScheme>
+    <a:fontScheme name="Office">
+      <a:majorFont>
+        <a:latin typeface="Arial" pitchFamily="0" charset="1"/>
+        <a:ea typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+        <a:cs typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+      </a:majorFont>
+      <a:minorFont>
+        <a:latin typeface="Arial" pitchFamily="0" charset="1"/>
+        <a:ea typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+        <a:cs typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+      </a:minorFont>
+    </a:fontScheme>
+    <a:fmtScheme>
+      <a:fillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:fillStyleLst>
+      <a:lnStyleLst>
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:prstDash val="solid"/>
+          <a:miter/>
+        </a:ln>
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:prstDash val="solid"/>
+          <a:miter/>
+        </a:ln>
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:prstDash val="solid"/>
+          <a:miter/>
+        </a:ln>
+      </a:lnStyleLst>
+      <a:effectStyleLst>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+      </a:effectStyleLst>
+      <a:bgFillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:bgFillStyleLst>
+    </a:fmtScheme>
+  </a:themeElements>
+</a:theme>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:F5"/>
   <sheetFormatPr defaultColWidth="11.55078125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="21.02"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="12.96"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="19.63"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="19.19"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="21.02"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="12.96"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="19.63"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="19.19"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="s">
+      <c r="A3" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="0" t="s">
+      <c r="B3" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="0" t="s">
+      <c r="C3" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="D3" s="0" t="s">
+      <c r="D3" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="E3" s="0" t="s">
+      <c r="E3" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="F3" s="0" t="s">
+      <c r="F3" s="1" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="s">
+      <c r="A4" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B4" s="2" t="n">
+      <c r="B4" s="3" t="n">
         <v>25</v>
       </c>
-      <c r="C4" s="2" t="n">
+      <c r="C4" s="3" t="n">
         <v>30</v>
       </c>
-      <c r="D4" s="0" t="n">
+      <c r="D4" s="1" t="n">
         <v>20</v>
       </c>
-      <c r="E4" s="2" t="n">
+      <c r="E4" s="3" t="n">
         <f aca="false">B4*D4</f>
         <v>500</v>
       </c>
-      <c r="F4" s="2" t="n">
+      <c r="F4" s="3" t="n">
         <f aca="false">C4*D4</f>
         <v>600</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="s">
+      <c r="A5" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="2" t="n">
+      <c r="B5" s="3" t="n">
         <v>100</v>
       </c>
-      <c r="C5" s="2" t="n">
+      <c r="C5" s="3" t="n">
         <v>90</v>
       </c>
-      <c r="D5" s="0" t="n">
+      <c r="D5" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="E5" s="2" t="n">
+      <c r="E5" s="3" t="n">
         <f aca="false">B5*D5</f>
         <v>100</v>
       </c>
-      <c r="F5" s="2" t="n">
+      <c r="F5" s="3" t="n">
         <f aca="false">C5*D5</f>
         <v>90</v>
       </c>
@@ -417,287 +526,227 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:F31"/>
   <sheetFormatPr defaultColWidth="11.55078125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="21.02"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="12.96"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="19.63"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="19.19"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="21.02"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="12.96"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="19.63"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="19.19"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="s">
+      <c r="A3" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="0" t="s">
+      <c r="B3" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="0" t="s">
+      <c r="C3" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="D3" s="0" t="s">
+      <c r="D3" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="E3" s="0" t="s">
+      <c r="E3" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="F3" s="0" t="s">
+      <c r="F3" s="1" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="s">
+      <c r="A4" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B4" s="2" t="n">
+      <c r="B4" s="3" t="n">
         <v>25</v>
       </c>
-      <c r="C4" s="2" t="n">
+      <c r="C4" s="3" t="n">
         <v>30</v>
       </c>
-      <c r="D4" s="0" t="n">
+      <c r="D4" s="1" t="n">
         <v>20</v>
       </c>
-      <c r="E4" s="2" t="n">
+      <c r="E4" s="3" t="n">
         <f aca="false">B4*D4</f>
         <v>500</v>
       </c>
-      <c r="F4" s="2" t="n">
+      <c r="F4" s="3" t="n">
         <f aca="false">C4*D4</f>
         <v>600</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="s">
+      <c r="A5" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="2" t="n">
+      <c r="B5" s="3" t="n">
         <v>100</v>
       </c>
-      <c r="C5" s="2" t="n">
+      <c r="C5" s="3" t="n">
         <v>90</v>
       </c>
-      <c r="D5" s="0" t="n">
+      <c r="D5" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="E5" s="2" t="n">
+      <c r="E5" s="3" t="n">
         <f aca="false">B5*D5</f>
         <v>100</v>
       </c>
-      <c r="F5" s="2" t="n">
+      <c r="F5" s="3" t="n">
         <f aca="false">C5*D5</f>
         <v>90</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="0" t="s">
+      <c r="A7" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B7" s="2" t="n">
+      <c r="B7" s="3" t="n">
         <v>1000000</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="3" t="s">
+      <c r="A9" s="4" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="0" t="s">
+      <c r="A10" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B10" s="0" t="n">
-        <f aca="false">B7/(B4+B5)</f>
-        <v>8000</v>
-      </c>
-      <c r="C10" s="0" t="s">
+      <c r="C10" s="1" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B11" s="4" t="n">
-        <f aca="false">B7/(B4+B5)</f>
-        <v>8000</v>
-      </c>
-      <c r="C11" s="0" t="s">
+      <c r="B11" s="5"/>
+      <c r="C11" s="1" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B12" s="2" t="n">
-        <f aca="false">B10*B4</f>
-        <v>200000</v>
-      </c>
-      <c r="C12" s="0" t="s">
+      <c r="B12" s="3"/>
+      <c r="C12" s="1" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B13" s="2" t="n">
-        <f aca="false">B11*B5</f>
-        <v>800000</v>
-      </c>
-      <c r="C13" s="0" t="s">
+      <c r="B13" s="3"/>
+      <c r="C13" s="1" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B14" s="5" t="n">
-        <f aca="false">B12/B7</f>
-        <v>0.2</v>
-      </c>
-      <c r="C14" s="0" t="s">
+      <c r="B14" s="6"/>
+      <c r="C14" s="1" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B15" s="5" t="n">
-        <f aca="false">B13/B7</f>
-        <v>0.8</v>
-      </c>
-      <c r="C15" s="0" t="s">
+      <c r="B15" s="6"/>
+      <c r="C15" s="1" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="0" t="s">
+      <c r="A16" s="1" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B17" s="2" t="n">
-        <f aca="false">B10*C4 + B11*C5</f>
-        <v>960000</v>
-      </c>
-      <c r="C17" s="0" t="s">
+      <c r="B17" s="3"/>
+      <c r="C17" s="1" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B18" s="6" t="n">
-        <f aca="false">B17/B7 - 1</f>
-        <v>-0.04</v>
-      </c>
-      <c r="C18" s="3" t="s">
+      <c r="B18" s="7"/>
+      <c r="C18" s="4" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="0" t="s">
+      <c r="A19" s="1" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B20" s="5" t="n">
-        <f aca="false">C4/B4-1</f>
-        <v>0.2</v>
-      </c>
-      <c r="C20" s="0" t="s">
+      <c r="B20" s="6"/>
+      <c r="C20" s="1" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B21" s="5" t="n">
-        <f aca="false">C5/B5-1</f>
-        <v>-0.1</v>
-      </c>
-      <c r="C21" s="0" t="s">
+      <c r="B21" s="6"/>
+      <c r="C21" s="1" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B22" s="6" t="n">
-        <f aca="false">B14*B20 + B15*B21</f>
-        <v>-0.04</v>
-      </c>
-      <c r="C22" s="3" t="s">
+      <c r="B22" s="7"/>
+      <c r="C22" s="4" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="0" t="s">
+      <c r="A23" s="1" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B24" s="5" t="n">
-        <f aca="false">C4/(C4+C5)</f>
-        <v>0.25</v>
-      </c>
-      <c r="C24" s="0" t="s">
+      <c r="B24" s="6"/>
+      <c r="C24" s="1" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B25" s="5" t="n">
-        <f aca="false">C5/(C4+C5)</f>
-        <v>0.75</v>
-      </c>
-      <c r="C25" s="0" t="s">
+      <c r="B25" s="6"/>
+      <c r="C25" s="1" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B26" s="0" t="n">
-        <f aca="false">B24*B17 / C4</f>
-        <v>8000</v>
-      </c>
-      <c r="C26" s="0" t="s">
+      <c r="C26" s="1" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B27" s="4" t="n">
-        <f aca="false">B25*B17 / C5</f>
-        <v>8000</v>
-      </c>
-      <c r="C27" s="0" t="s">
+      <c r="B27" s="5"/>
+      <c r="C27" s="1" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B28" s="7" t="n">
-        <f aca="false">C4*(B26 - B10)</f>
-        <v>0</v>
-      </c>
-      <c r="C28" s="4" t="s">
+      <c r="B28" s="8"/>
+      <c r="C28" s="5" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B29" s="7" t="n">
-        <f aca="false">C5*(B27 - B11)</f>
-        <v>0</v>
-      </c>
-      <c r="C29" s="4" t="s">
+      <c r="B29" s="8"/>
+      <c r="C29" s="5" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B30" s="8" t="n">
-        <f aca="false">ABS(B28) + ABS(B29)</f>
-        <v>0</v>
-      </c>
-      <c r="C30" s="3" t="s">
+      <c r="B30" s="9"/>
+      <c r="C30" s="4" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B31" s="0" t="n">
-        <f aca="false">B30/B7</f>
-        <v>0</v>
-      </c>
-      <c r="C31" s="0" t="s">
+      <c r="C31" s="1" t="s">
         <v>33</v>
       </c>
     </row>
@@ -713,285 +762,230 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:F32"/>
   <sheetFormatPr defaultColWidth="11.55078125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="21.02"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="12.96"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="19.63"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="19.19"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="21.02"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="12.96"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="19.63"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="19.19"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="s">
+      <c r="A3" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="0" t="s">
+      <c r="B3" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="0" t="s">
+      <c r="C3" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="D3" s="0" t="s">
+      <c r="D3" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="E3" s="0" t="s">
+      <c r="E3" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="F3" s="0" t="s">
+      <c r="F3" s="1" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="s">
+      <c r="A4" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B4" s="2" t="n">
+      <c r="B4" s="3" t="n">
         <v>25</v>
       </c>
-      <c r="C4" s="2" t="n">
+      <c r="C4" s="3" t="n">
         <v>30</v>
       </c>
-      <c r="D4" s="0" t="n">
+      <c r="D4" s="1" t="n">
         <v>20</v>
       </c>
-      <c r="E4" s="2" t="n">
+      <c r="E4" s="3" t="n">
         <f aca="false">B4*D4</f>
         <v>500</v>
       </c>
-      <c r="F4" s="2" t="n">
+      <c r="F4" s="3" t="n">
         <f aca="false">C4*D4</f>
         <v>600</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="s">
+      <c r="A5" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="2" t="n">
+      <c r="B5" s="3" t="n">
         <v>100</v>
       </c>
-      <c r="C5" s="2" t="n">
+      <c r="C5" s="3" t="n">
         <v>90</v>
       </c>
-      <c r="D5" s="0" t="n">
+      <c r="D5" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="E5" s="2" t="n">
+      <c r="E5" s="3" t="n">
         <f aca="false">B5*D5</f>
         <v>100</v>
       </c>
-      <c r="F5" s="2" t="n">
+      <c r="F5" s="3" t="n">
         <f aca="false">C5*D5</f>
         <v>90</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="0" t="s">
+      <c r="A7" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B7" s="2" t="n">
+      <c r="B7" s="3" t="n">
         <v>1000000</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="3" t="s">
+      <c r="A9" s="4" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="0" t="s">
+      <c r="A10" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B10" s="5" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="C10" s="0" t="s">
+      <c r="B10" s="6"/>
+      <c r="C10" s="1" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="3"/>
-      <c r="B11" s="5" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="C11" s="0" t="s">
+      <c r="A11" s="4"/>
+      <c r="B11" s="6"/>
+      <c r="C11" s="1" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B12" s="2" t="n">
-        <f aca="false">B7*B10</f>
-        <v>500000</v>
-      </c>
-      <c r="C12" s="0" t="s">
+      <c r="B12" s="3"/>
+      <c r="C12" s="1" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="3"/>
-      <c r="B13" s="2" t="n">
-        <f aca="false">B7*B11</f>
-        <v>500000</v>
-      </c>
-      <c r="C13" s="0" t="s">
+      <c r="A13" s="4"/>
+      <c r="B13" s="3"/>
+      <c r="C13" s="1" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B14" s="0" t="n">
-        <f aca="false">B12 / B4</f>
-        <v>20000</v>
-      </c>
-      <c r="C14" s="0" t="s">
+      <c r="C14" s="1" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B15" s="0" t="n">
-        <f aca="false">B13 / B5</f>
-        <v>5000</v>
-      </c>
-      <c r="C15" s="0" t="s">
+      <c r="C15" s="1" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="0" t="s">
+      <c r="A17" s="1" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B18" s="2" t="n">
-        <f aca="false">B14*C4 + B15*C5</f>
-        <v>1050000</v>
-      </c>
-      <c r="C18" s="0" t="s">
+      <c r="B18" s="3"/>
+      <c r="C18" s="1" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B19" s="6" t="n">
-        <f aca="false">B18/B7 - 1</f>
-        <v>0.05</v>
-      </c>
-      <c r="C19" s="3" t="s">
+      <c r="B19" s="7"/>
+      <c r="C19" s="4" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="0" t="s">
+      <c r="A20" s="1" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B21" s="5" t="n">
-        <f aca="false">C4/B4-1</f>
-        <v>0.2</v>
-      </c>
-      <c r="C21" s="0" t="s">
+      <c r="B21" s="6"/>
+      <c r="C21" s="1" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B22" s="5" t="n">
-        <f aca="false">C5/B5-1</f>
-        <v>-0.1</v>
-      </c>
-      <c r="C22" s="0" t="s">
+      <c r="B22" s="6"/>
+      <c r="C22" s="1" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B23" s="6" t="n">
-        <f aca="false">B10*B21 + B11*B22</f>
-        <v>0.05</v>
-      </c>
-      <c r="C23" s="3" t="s">
+      <c r="B23" s="7"/>
+      <c r="C23" s="4" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="0" t="s">
+      <c r="A24" s="1" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B25" s="5" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="C25" s="0" t="s">
+      <c r="B25" s="6"/>
+      <c r="C25" s="1" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B26" s="5" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="C26" s="0" t="s">
+      <c r="B26" s="6"/>
+      <c r="C26" s="1" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B27" s="9" t="n">
-        <f aca="false">B25*B18 / C4</f>
-        <v>17500</v>
-      </c>
-      <c r="C27" s="0" t="s">
+      <c r="B27" s="10"/>
+      <c r="C27" s="1" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B28" s="10" t="n">
-        <f aca="false">B26*B18 / C5</f>
-        <v>5833.33333333333</v>
-      </c>
-      <c r="C28" s="0" t="s">
+      <c r="B28" s="11"/>
+      <c r="C28" s="1" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B29" s="7" t="n">
-        <f aca="false">C4*(B27 - B14)</f>
-        <v>-75000</v>
-      </c>
-      <c r="C29" s="4" t="s">
+      <c r="B29" s="8"/>
+      <c r="C29" s="5" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B30" s="7" t="n">
-        <f aca="false">C5*(B28 - B15)</f>
-        <v>75000</v>
-      </c>
-      <c r="C30" s="4" t="s">
+      <c r="B30" s="8"/>
+      <c r="C30" s="5" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B31" s="8" t="n">
-        <f aca="false">ABS(B29) + ABS(B30)</f>
-        <v>150000</v>
-      </c>
-      <c r="C31" s="3" t="s">
+      <c r="B31" s="9"/>
+      <c r="C31" s="4" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B32" s="5" t="n">
-        <f aca="false">B31/B7</f>
-        <v>0.15</v>
-      </c>
-      <c r="C32" s="0" t="s">
+      <c r="B32" s="6"/>
+      <c r="C32" s="1" t="s">
         <v>33</v>
       </c>
     </row>
@@ -1007,289 +1001,232 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:F32"/>
   <sheetFormatPr defaultColWidth="11.55078125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="21.02"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="12.96"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="19.63"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="19.19"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="21.02"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="12.96"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="19.63"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="19.19"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="s">
+      <c r="A3" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="0" t="s">
+      <c r="B3" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="0" t="s">
+      <c r="C3" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="D3" s="0" t="s">
+      <c r="D3" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="E3" s="0" t="s">
+      <c r="E3" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="F3" s="0" t="s">
+      <c r="F3" s="1" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="s">
+      <c r="A4" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B4" s="2" t="n">
+      <c r="B4" s="3" t="n">
         <v>25</v>
       </c>
-      <c r="C4" s="2" t="n">
+      <c r="C4" s="3" t="n">
         <v>30</v>
       </c>
-      <c r="D4" s="0" t="n">
+      <c r="D4" s="1" t="n">
         <v>20</v>
       </c>
-      <c r="E4" s="2" t="n">
+      <c r="E4" s="3" t="n">
         <f aca="false">B4*D4</f>
         <v>500</v>
       </c>
-      <c r="F4" s="2" t="n">
+      <c r="F4" s="3" t="n">
         <f aca="false">C4*D4</f>
         <v>600</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="s">
+      <c r="A5" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="2" t="n">
+      <c r="B5" s="3" t="n">
         <v>100</v>
       </c>
-      <c r="C5" s="2" t="n">
+      <c r="C5" s="3" t="n">
         <v>90</v>
       </c>
-      <c r="D5" s="0" t="n">
+      <c r="D5" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="E5" s="2" t="n">
+      <c r="E5" s="3" t="n">
         <f aca="false">B5*D5</f>
         <v>100</v>
       </c>
-      <c r="F5" s="2" t="n">
+      <c r="F5" s="3" t="n">
         <f aca="false">C5*D5</f>
         <v>90</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="0" t="s">
+      <c r="A7" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="B7" s="2" t="n">
+      <c r="B7" s="3" t="n">
         <v>1000000</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="3" t="s">
+      <c r="A9" s="4" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="0" t="s">
+      <c r="A10" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B10" s="5" t="n">
-        <f aca="false">E4/(E4+E5)</f>
-        <v>0.833333333333333</v>
-      </c>
-      <c r="C10" s="0" t="s">
+      <c r="B10" s="6"/>
+      <c r="C10" s="1" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="3"/>
-      <c r="B11" s="5" t="n">
-        <f aca="false">E5/(E4+E5)</f>
-        <v>0.166666666666667</v>
-      </c>
-      <c r="C11" s="0" t="s">
+      <c r="A11" s="4"/>
+      <c r="B11" s="6"/>
+      <c r="C11" s="1" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B12" s="2" t="n">
-        <f aca="false">B7*B10</f>
-        <v>833333.333333333</v>
-      </c>
-      <c r="C12" s="0" t="s">
+      <c r="B12" s="3"/>
+      <c r="C12" s="1" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="3"/>
-      <c r="B13" s="2" t="n">
-        <f aca="false">B7*B11</f>
-        <v>166666.666666667</v>
-      </c>
-      <c r="C13" s="0" t="s">
+      <c r="A13" s="4"/>
+      <c r="B13" s="3"/>
+      <c r="C13" s="1" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B14" s="9" t="n">
-        <f aca="false">B12 / B4</f>
-        <v>33333.3333333333</v>
-      </c>
-      <c r="C14" s="0" t="s">
+      <c r="B14" s="10"/>
+      <c r="C14" s="1" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B15" s="9" t="n">
-        <f aca="false">B13 / B5</f>
-        <v>1666.66666666667</v>
-      </c>
-      <c r="C15" s="0" t="s">
+      <c r="B15" s="10"/>
+      <c r="C15" s="1" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="0" t="s">
+      <c r="A17" s="1" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B18" s="2" t="n">
-        <f aca="false">B14*C4 + B15*C5</f>
-        <v>1150000</v>
-      </c>
-      <c r="C18" s="0" t="s">
+      <c r="B18" s="3"/>
+      <c r="C18" s="1" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B19" s="6" t="n">
-        <f aca="false">B18/B7 - 1</f>
-        <v>0.15</v>
-      </c>
-      <c r="C19" s="3" t="s">
+      <c r="B19" s="7"/>
+      <c r="C19" s="4" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="0" t="s">
+      <c r="A20" s="1" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B21" s="5" t="n">
-        <f aca="false">C4/B4-1</f>
-        <v>0.2</v>
-      </c>
-      <c r="C21" s="0" t="s">
+      <c r="B21" s="6"/>
+      <c r="C21" s="1" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B22" s="5" t="n">
-        <f aca="false">C5/B5-1</f>
-        <v>-0.1</v>
-      </c>
-      <c r="C22" s="0" t="s">
+      <c r="B22" s="6"/>
+      <c r="C22" s="1" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B23" s="6" t="n">
-        <f aca="false">B10*B21 + B11*B22</f>
-        <v>0.15</v>
-      </c>
-      <c r="C23" s="3" t="s">
+      <c r="B23" s="7"/>
+      <c r="C23" s="4" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="0" t="s">
+      <c r="A24" s="1" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B25" s="5" t="n">
-        <f aca="false">F4/(F4+F5)</f>
-        <v>0.869565217391304</v>
-      </c>
-      <c r="C25" s="0" t="s">
+      <c r="B25" s="6"/>
+      <c r="C25" s="1" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B26" s="5" t="n">
-        <f aca="false">F5/(F4+F5)</f>
-        <v>0.130434782608696</v>
-      </c>
-      <c r="C26" s="0" t="s">
+      <c r="B26" s="6"/>
+      <c r="C26" s="1" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B27" s="9" t="n">
-        <f aca="false">B25*B18 / C4</f>
-        <v>33333.3333333333</v>
-      </c>
-      <c r="C27" s="0" t="s">
+      <c r="B27" s="10"/>
+      <c r="C27" s="1" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B28" s="10" t="n">
-        <f aca="false">B26*B18 / C5</f>
-        <v>1666.66666666667</v>
-      </c>
-      <c r="C28" s="0" t="s">
+      <c r="B28" s="11"/>
+      <c r="C28" s="1" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B29" s="7" t="n">
-        <f aca="false">C4*(B27 - B14)</f>
-        <v>0</v>
-      </c>
-      <c r="C29" s="4" t="s">
+      <c r="B29" s="8"/>
+      <c r="C29" s="5" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B30" s="7" t="n">
-        <f aca="false">C5*(B28 - B15)</f>
-        <v>0</v>
-      </c>
-      <c r="C30" s="4" t="s">
+      <c r="B30" s="8"/>
+      <c r="C30" s="5" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B31" s="8" t="n">
-        <f aca="false">ABS(B29) + ABS(B30)</f>
-        <v>0</v>
-      </c>
-      <c r="C31" s="3" t="s">
+      <c r="B31" s="9"/>
+      <c r="C31" s="4" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B32" s="5" t="n">
-        <f aca="false">B31/B7</f>
-        <v>0</v>
-      </c>
-      <c r="C32" s="0" t="s">
+      <c r="B32" s="6"/>
+      <c r="C32" s="1" t="s">
         <v>33</v>
       </c>
     </row>
@@ -1305,140 +1242,123 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:F14"/>
   <sheetFormatPr defaultColWidth="11.55078125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="19.63"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="19.19"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="19.63"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="19.19"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="12" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="s">
+      <c r="A3" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="0" t="s">
+      <c r="B3" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="0" t="s">
+      <c r="C3" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="D3" s="0" t="s">
+      <c r="D3" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="E3" s="0" t="s">
+      <c r="E3" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="F3" s="0" t="s">
+      <c r="F3" s="1" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="s">
+      <c r="A4" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B4" s="2" t="n">
+      <c r="B4" s="3" t="n">
         <v>25</v>
       </c>
-      <c r="C4" s="2" t="n">
+      <c r="C4" s="3" t="n">
         <v>30</v>
       </c>
-      <c r="D4" s="0" t="n">
+      <c r="D4" s="1" t="n">
         <v>20</v>
       </c>
-      <c r="E4" s="2" t="n">
+      <c r="E4" s="3" t="n">
         <f aca="false">B4*D4</f>
         <v>500</v>
       </c>
-      <c r="F4" s="2" t="n">
+      <c r="F4" s="3" t="n">
         <f aca="false">C4*D4</f>
         <v>600</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="s">
+      <c r="A5" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="2" t="n">
+      <c r="B5" s="3" t="n">
         <v>100</v>
       </c>
-      <c r="C5" s="2" t="n">
+      <c r="C5" s="3" t="n">
         <v>90</v>
       </c>
-      <c r="D5" s="0" t="n">
+      <c r="D5" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="E5" s="2" t="n">
+      <c r="E5" s="3" t="n">
         <f aca="false">B5*D5</f>
         <v>100</v>
       </c>
-      <c r="F5" s="2" t="n">
+      <c r="F5" s="3" t="n">
         <f aca="false">C5*D5</f>
         <v>90</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="0" t="s">
+      <c r="A7" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="C7" s="0" t="n">
-        <v>6</v>
-      </c>
+      <c r="C7" s="1"/>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="0" t="s">
+      <c r="A8" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="C8" s="0" t="n">
-        <f aca="false">(E4+E5)/C7</f>
-        <v>100</v>
-      </c>
+      <c r="C8" s="1"/>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="0" t="s">
+      <c r="A10" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="C10" s="0" t="n">
-        <f aca="false">C7</f>
-        <v>6</v>
-      </c>
-      <c r="D10" s="2"/>
+      <c r="C10" s="1"/>
+      <c r="D10" s="3"/>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="0" t="s">
+      <c r="A11" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="C11" s="0" t="n">
-        <f aca="false">(F4+F5)/C10</f>
-        <v>115</v>
-      </c>
-      <c r="D11" s="2"/>
+      <c r="C11" s="1"/>
+      <c r="D11" s="3"/>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="0" t="s">
+      <c r="A13" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="C13" s="5" t="n">
-        <f aca="false">C11/C8-1</f>
-        <v>0.15</v>
-      </c>
+      <c r="C13" s="6"/>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="0" t="s">
+      <c r="A14" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="C14" s="5" t="n">
-        <f aca="false">'Example 3 - Value weighting'!B19</f>
-        <v>0.15</v>
-      </c>
+      <c r="C14" s="6"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>